<commit_message>
Unify ticket layout and refine candidate contexts and workspace styling
</commit_message>
<xml_diff>
--- a/PROJECTS_EXCEL/workbook/cfgDependencies.xlsx
+++ b/PROJECTS_EXCEL/workbook/cfgDependencies.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\WORK\Windows\Projects\ExcelPrototype\PROJECTS_EXCEL\workbook\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1AEE71C-A6BF-4683-9638-666806399709}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A17C11B8-B10A-4B05-A06F-4270174101A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -414,9 +414,6 @@
     <t>tbTickets::column.out_food</t>
   </si>
   <si>
-    <t>Вибуття.Продовольче</t>
-  </si>
-  <si>
     <t>tbTickets::column.position</t>
   </si>
   <si>
@@ -550,6 +547,9 @@
   </si>
   <si>
     <t>[Посади$A1:E12000]</t>
+  </si>
+  <si>
+    <t>Вибуття.ПЗ</t>
   </si>
 </sst>
 </file>
@@ -2017,7 +2017,7 @@
         <v>127</v>
       </c>
       <c r="D66" s="8" t="s">
-        <v>128</v>
+        <v>173</v>
       </c>
     </row>
     <row r="67" spans="2:4" ht="18.75" x14ac:dyDescent="0.25">
@@ -2025,10 +2025,10 @@
         <v>107</v>
       </c>
       <c r="C67" s="7" t="s">
+        <v>128</v>
+      </c>
+      <c r="D67" s="8" t="s">
         <v>129</v>
-      </c>
-      <c r="D67" s="8" t="s">
-        <v>130</v>
       </c>
     </row>
     <row r="68" spans="2:4" ht="18.75" x14ac:dyDescent="0.25">
@@ -2036,10 +2036,10 @@
         <v>107</v>
       </c>
       <c r="C68" s="7" t="s">
+        <v>130</v>
+      </c>
+      <c r="D68" s="8" t="s">
         <v>131</v>
-      </c>
-      <c r="D68" s="8" t="s">
-        <v>132</v>
       </c>
     </row>
     <row r="69" spans="2:4" ht="18.75" x14ac:dyDescent="0.25">
@@ -2047,10 +2047,10 @@
         <v>107</v>
       </c>
       <c r="C69" s="7" t="s">
+        <v>132</v>
+      </c>
+      <c r="D69" s="8" t="s">
         <v>133</v>
-      </c>
-      <c r="D69" s="8" t="s">
-        <v>134</v>
       </c>
     </row>
     <row r="70" spans="2:4" ht="18.75" x14ac:dyDescent="0.25">
@@ -2058,10 +2058,10 @@
         <v>107</v>
       </c>
       <c r="C70" s="7" t="s">
+        <v>134</v>
+      </c>
+      <c r="D70" s="8" t="s">
         <v>135</v>
-      </c>
-      <c r="D70" s="8" t="s">
-        <v>136</v>
       </c>
     </row>
     <row r="71" spans="2:4" ht="18.75" x14ac:dyDescent="0.25">
@@ -2069,10 +2069,10 @@
         <v>107</v>
       </c>
       <c r="C71" s="7" t="s">
+        <v>136</v>
+      </c>
+      <c r="D71" s="8" t="s">
         <v>137</v>
-      </c>
-      <c r="D71" s="8" t="s">
-        <v>138</v>
       </c>
     </row>
     <row r="72" spans="2:4" ht="18.75" x14ac:dyDescent="0.25">
@@ -2080,32 +2080,32 @@
         <v>6</v>
       </c>
       <c r="C72" s="7" t="s">
+        <v>138</v>
+      </c>
+      <c r="D72" s="8" t="s">
         <v>139</v>
-      </c>
-      <c r="D72" s="8" t="s">
-        <v>140</v>
       </c>
     </row>
     <row r="73" spans="2:4" ht="18.75" x14ac:dyDescent="0.25">
       <c r="B73" s="6" t="s">
+        <v>140</v>
+      </c>
+      <c r="C73" s="7" t="s">
         <v>141</v>
       </c>
-      <c r="C73" s="7" t="s">
+      <c r="D73" s="8" t="s">
         <v>142</v>
-      </c>
-      <c r="D73" s="8" t="s">
-        <v>143</v>
       </c>
     </row>
     <row r="74" spans="2:4" ht="18.75" x14ac:dyDescent="0.25">
       <c r="B74" s="6" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C74" s="7" t="s">
+        <v>143</v>
+      </c>
+      <c r="D74" s="8" t="s">
         <v>144</v>
-      </c>
-      <c r="D74" s="8" t="s">
-        <v>145</v>
       </c>
     </row>
     <row r="75" spans="2:4" ht="18.75" x14ac:dyDescent="0.25">
@@ -2113,10 +2113,10 @@
         <v>9</v>
       </c>
       <c r="C75" s="7" t="s">
+        <v>145</v>
+      </c>
+      <c r="D75" s="8" t="s">
         <v>146</v>
-      </c>
-      <c r="D75" s="8" t="s">
-        <v>147</v>
       </c>
     </row>
     <row r="76" spans="2:4" ht="18.75" x14ac:dyDescent="0.25">
@@ -2124,10 +2124,10 @@
         <v>9</v>
       </c>
       <c r="C76" s="7" t="s">
+        <v>147</v>
+      </c>
+      <c r="D76" s="8" t="s">
         <v>148</v>
-      </c>
-      <c r="D76" s="8" t="s">
-        <v>149</v>
       </c>
     </row>
     <row r="77" spans="2:4" ht="18.75" x14ac:dyDescent="0.25">
@@ -2135,10 +2135,10 @@
         <v>9</v>
       </c>
       <c r="C77" s="7" t="s">
+        <v>149</v>
+      </c>
+      <c r="D77" s="8" t="s">
         <v>150</v>
-      </c>
-      <c r="D77" s="8" t="s">
-        <v>151</v>
       </c>
     </row>
     <row r="78" spans="2:4" ht="18.75" x14ac:dyDescent="0.25">
@@ -2146,10 +2146,10 @@
         <v>9</v>
       </c>
       <c r="C78" s="7" t="s">
+        <v>151</v>
+      </c>
+      <c r="D78" s="8" t="s">
         <v>152</v>
-      </c>
-      <c r="D78" s="8" t="s">
-        <v>153</v>
       </c>
     </row>
     <row r="79" spans="2:4" ht="18.75" x14ac:dyDescent="0.25">
@@ -2157,10 +2157,10 @@
         <v>9</v>
       </c>
       <c r="C79" s="7" t="s">
+        <v>153</v>
+      </c>
+      <c r="D79" s="8" t="s">
         <v>154</v>
-      </c>
-      <c r="D79" s="8" t="s">
-        <v>155</v>
       </c>
     </row>
     <row r="80" spans="2:4" ht="18.75" x14ac:dyDescent="0.25">
@@ -2168,21 +2168,21 @@
         <v>6</v>
       </c>
       <c r="C80" s="7" t="s">
+        <v>155</v>
+      </c>
+      <c r="D80" s="8" t="s">
         <v>156</v>
-      </c>
-      <c r="D80" s="8" t="s">
-        <v>157</v>
       </c>
     </row>
     <row r="81" spans="2:4" ht="18.75" x14ac:dyDescent="0.25">
       <c r="B81" s="6" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C81" s="7" t="s">
+        <v>157</v>
+      </c>
+      <c r="D81" s="8" t="s">
         <v>158</v>
-      </c>
-      <c r="D81" s="8" t="s">
-        <v>159</v>
       </c>
     </row>
     <row r="82" spans="2:4" ht="18.75" x14ac:dyDescent="0.25">
@@ -2190,21 +2190,21 @@
         <v>6</v>
       </c>
       <c r="C82" s="7" t="s">
+        <v>159</v>
+      </c>
+      <c r="D82" s="8" t="s">
         <v>160</v>
-      </c>
-      <c r="D82" s="8" t="s">
-        <v>161</v>
       </c>
     </row>
     <row r="83" spans="2:4" ht="18.75" x14ac:dyDescent="0.25">
       <c r="B83" s="6" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C83" s="7" t="s">
+        <v>161</v>
+      </c>
+      <c r="D83" s="8" t="s">
         <v>162</v>
-      </c>
-      <c r="D83" s="8" t="s">
-        <v>163</v>
       </c>
     </row>
     <row r="84" spans="2:4" ht="18.75" x14ac:dyDescent="0.25">
@@ -2212,7 +2212,7 @@
         <v>107</v>
       </c>
       <c r="C84" s="7" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="D84" s="8" t="s">
         <v>49</v>
@@ -2223,7 +2223,7 @@
         <v>107</v>
       </c>
       <c r="C85" s="7" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="D85" s="8" t="s">
         <v>51</v>
@@ -2234,10 +2234,10 @@
         <v>6</v>
       </c>
       <c r="C86" s="7" t="s">
+        <v>165</v>
+      </c>
+      <c r="D86" s="8" t="s">
         <v>166</v>
-      </c>
-      <c r="D86" s="8" t="s">
-        <v>167</v>
       </c>
     </row>
     <row r="87" spans="2:4" ht="18.75" x14ac:dyDescent="0.25">
@@ -2245,32 +2245,32 @@
         <v>6</v>
       </c>
       <c r="C87" s="7" t="s">
+        <v>167</v>
+      </c>
+      <c r="D87" s="8" t="s">
         <v>168</v>
-      </c>
-      <c r="D87" s="8" t="s">
-        <v>169</v>
       </c>
     </row>
     <row r="88" spans="2:4" ht="18.75" x14ac:dyDescent="0.25">
       <c r="B88" s="6" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C88" s="7" t="s">
+        <v>169</v>
+      </c>
+      <c r="D88" s="8" t="s">
         <v>170</v>
-      </c>
-      <c r="D88" s="8" t="s">
-        <v>171</v>
       </c>
     </row>
     <row r="89" spans="2:4" ht="18.75" x14ac:dyDescent="0.25">
       <c r="B89" s="6" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C89" s="7" t="s">
+        <v>171</v>
+      </c>
+      <c r="D89" s="8" t="s">
         <v>172</v>
-      </c>
-      <c r="D89" s="8" t="s">
-        <v>173</v>
       </c>
     </row>
   </sheetData>

</xml_diff>